<commit_message>
Photo audit round 3: stop pending_review leaks in 4 query paths
Pending_review photos (review-before-process workflow) were leaking into
queries that should treat them as not-yet-existing. NULL-safe exclusion
via .or() since Postgres .neq excludes NULL rows.

- audit/photos: 'all' and 'untagged' zones excluded pending_review
- reports/unreported: report composer was offering pending photos
- reports/available-photos: same
- parent/photos: parents could see pre-review captures
</commit_message>
<xml_diff>
--- a/Montree_Master_Outreach.xlsx
+++ b/Montree_Master_Outreach.xlsx
@@ -8,12 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Global Outreach (420)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="China Montessori (303)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="China Montessori (350)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Global Outreach (420)'!$A$1:$K$421</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'China Montessori (303)'!$A$1:$I$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'China Montessori (350)'!$A$1:$I$303</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -22006,7 +22006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I303"/>
+  <dimension ref="A1:I351"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="45" customWidth="1" style="11" min="1" max="1"/>
@@ -32567,6 +32567,1614 @@
           <t>Montessori</t>
         </is>
       </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>新颖(蒙特梭利)幼儿园</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Dalian</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>开发区金桥花园金湖里小区33号</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>0411-87612992/13390505867</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr"/>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>阳光艺蒙幼儿园</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Dalian</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>大连市金州区舒林园</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr"/>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="inlineStr"/>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>邦贝泽石幼儿园</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Dalian</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>辽宁省大连市甘井子区虹霞路197-6号</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>0411-39506389/18100423311</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr"/>
+      <c r="G306" t="inlineStr"/>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>甘井子区万科假日风景幼儿园</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Dalian</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>辽宁省大连市甘井子区红旗西路104-6号</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr"/>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>爱博雅北岸自然教育幼儿园</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Dalian</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>辽宁省大连市金州区钢铁路鹏程家园31号楼</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr"/>
+      <c r="F308" t="inlineStr"/>
+      <c r="G308" t="inlineStr"/>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>启蒙幼儿娱乐园</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Dalian</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>辽宁省大连市西岗区沈铁·站北新居D区</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>13500783822</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr"/>
+      <c r="G309" t="inlineStr"/>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>玛利娅蒙特梭利爱与自由幼儿园</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Harbin</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Heilongjiang</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>黑龙江省哈尔滨市南岗区渭水路24号</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr"/>
+      <c r="F310" t="inlineStr"/>
+      <c r="G310" t="inlineStr"/>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>蒙台梭利教育</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Harbin</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Heilongjiang</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>哈尔滨市道里区顾新路康安家园</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr"/>
+      <c r="F311" t="inlineStr"/>
+      <c r="G311" t="inlineStr"/>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>莱恩蒙特梭利幼儿教育</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Changchun</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Jilin</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>长春市绿园区万达华府B1-2-138室</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>15944007200</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr"/>
+      <c r="G312" t="inlineStr"/>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>莲上蒙台梭利幼儿园</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Changchun</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Jilin</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>吉林省长春市绿园区腾飞大道305号恒大首府首期</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>18666602014</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="inlineStr"/>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>长春市南关区蒙爱童幼儿园</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Changchun</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Jilin</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>吉林省长春市南关区东岭南街1090号</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>0431-88413488</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr"/>
+      <c r="G314" t="inlineStr"/>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>蒙特梭利巴顿国际早教中心</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Changchun</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Jilin</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>吉林省长春市绿园区西安大路5330号</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr"/>
+      <c r="F315" t="inlineStr"/>
+      <c r="G315" t="inlineStr"/>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>无锡市嘉德琳蒙台梭利幼儿园</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Wuxi</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>无锡市滨湖区中南西路399号（蠡湖香樟园内）</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>0510-82860536</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr"/>
+      <c r="G316" t="inlineStr"/>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>无锡市滨湖区蒙淇星实验幼儿园</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Wuxi</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>无锡市滨湖区唐巷路8号</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>15371056123</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="inlineStr"/>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>太原市古交市童恩幼儿园·蒙特梭利</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Taiyuan</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Shanxi</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>太原市古交市金刚堰路68号</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr"/>
+      <c r="F318" t="inlineStr"/>
+      <c r="G318" t="inlineStr"/>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>富华松竹六一蒙台梭利实验幼儿园</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Guiyang</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Guizhou</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>贵州省贵阳市南明区红岩路78号</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>0851-85372702</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr"/>
+      <c r="G319" t="inlineStr"/>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>伊顿慧智蒙台梭利幼儿园</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Nanning</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Guangxi</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>广西南宁市青秀区荣和大地校园</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr"/>
+      <c r="F320" t="inlineStr"/>
+      <c r="G320" t="inlineStr"/>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>格林贝恩蒙氏国际幼儿园</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Urumqi</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Xinjiang</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>新疆乌鲁木齐市新市区莉雨山南路金色家园社区</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr"/>
+      <c r="F321" t="inlineStr"/>
+      <c r="G321" t="inlineStr"/>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>金太阳幼儿园</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Wenzhou</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Zhejiang</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>浙江省温州市文成县泗溪河畔</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr"/>
+      <c r="F322" t="inlineStr"/>
+      <c r="G322" t="inlineStr"/>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>兴华蒙特梭利中英文幼儿园</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Zhuhai</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>广东省珠海市</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr"/>
+      <c r="F323" t="inlineStr"/>
+      <c r="G323" t="inlineStr"/>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>美好开端幼儿园</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Nanning</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Guangxi</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>广西壮族自治区南宁市西乡塘区秀厢大道81号保利爱琴海b108号</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>19163792454</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr"/>
+      <c r="G324" t="inlineStr"/>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>涵雅双语幼儿园</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Nanning</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Guangxi</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>广西壮族自治区南宁市西乡塘区友爱北路23-2号</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>13471198590/19968185986</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr"/>
+      <c r="G325" t="inlineStr"/>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>思维特国际双语幼儿园</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Guiyang</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Guizhou</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>贵州省贵阳市观山湖区石龙路190号</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>13312244172/13312244173</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr"/>
+      <c r="G326" t="inlineStr"/>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>艾贝尔中英文启蒙幼儿园</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Guiyang</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Guizhou</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>贵州省贵阳市白云区龚家寨街道X160</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>0851-84439813</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr"/>
+      <c r="G327" t="inlineStr"/>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>颂大童心爱尔贝蒙台梭利幼儿园</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Haikou</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Hainan</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>海南省海口市琼山区椰海大道13号</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>0898-65861211/13876334162</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr"/>
+      <c r="G328" t="inlineStr"/>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>琼山区爱尔贝蒙台梭利园</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Haikou</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Hainan</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>海口市琼山区椰航路</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr"/>
+      <c r="G329" t="inlineStr"/>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>蒙特梭利儿童成长中心(新城吾悦广场店)</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Haikou</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Hainan</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>海南省海口市龙华区美高街新城吾悦广场</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr"/>
+      <c r="F330" t="inlineStr"/>
+      <c r="G330" t="inlineStr"/>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>可宜蒙特梭利美国MIA认证早教托育</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Haikou</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Hainan</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>海南省海口市龙华区海德路9号现代花园D型2号楼S19号二楼</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>13876682806</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr"/>
+      <c r="G331" t="inlineStr"/>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>滨江海岸幼儿园</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Haikou</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Hainan</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>海南省海口市美兰区海甸一东路21-1号</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>13707517122</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr"/>
+      <c r="G332" t="inlineStr"/>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>欧范儿童世家奥北校区</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Shijiazhuang</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Hebei</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>河北省石家庄市长安区丰收路奥北公元一期8号楼</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>0311-67962338/15176872227</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr"/>
+      <c r="G333" t="inlineStr"/>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>润蒙·蒙特梭利托育中心</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Shijiazhuang</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Hebei</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>石家庄市裕华区东王街天海誉天下</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr"/>
+      <c r="F334" t="inlineStr"/>
+      <c r="G334" t="inlineStr"/>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>蒙特梭利儿童成长中心(海悦天地店)</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Shijiazhuang</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Hebei</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>河北省石家庄市桥西区裕华西路66号海悦天地购物广场F1</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr"/>
+      <c r="F335" t="inlineStr"/>
+      <c r="G335" t="inlineStr"/>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>萌然幼儿园</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Dongguan</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>广东省东莞市太宝路8号万科美好生活体验馆3层</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>13326894226/13377741821</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr"/>
+      <c r="G336" t="inlineStr"/>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>卡琳贝尔蒙台梭利幼儿园</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Dongguan</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>广东省东莞市虎门大道132号能源华庄A幢3楼</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>0769-85231366</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr"/>
+      <c r="G337" t="inlineStr"/>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>萌然蒙特梭利儿童成长基地</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Dongguan</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>广东省东莞市太宝路8号万科大都会3层</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>18825825502</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr"/>
+      <c r="G338" t="inlineStr"/>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>东莞市虎门乐辉生态幼儿园</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Dongguan</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>广东省东莞市五马1号</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr"/>
+      <c r="G339" t="inlineStr"/>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>蒙特梭利儿童成长中心(东田中心)</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Dongguan</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>广东省东莞市丽湖大道东田丽园会所二楼</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>0769-83827556/15024033150</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr"/>
+      <c r="G340" t="inlineStr"/>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>明日之星新桂幼儿园</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Foshan</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>佛山市顺德区新桂中路</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>18928635668</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr"/>
+      <c r="G341" t="inlineStr"/>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>明日之星蒙特梭利实验园(云盛路)</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Foshan</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>广东省佛山市顺德区云盛路十一街十巷2号</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>0757-22916363</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr"/>
+      <c r="G342" t="inlineStr"/>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>蒲公英蒙特梭利实验园(三月花分园)</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Foshan</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>广东省佛山市顺德区聚源直街四巷13号</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>0757-22225251</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr"/>
+      <c r="G343" t="inlineStr"/>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>蒲公英蒙特梭利实验园(五月花分园)</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Foshan</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>广东省佛山市顺德区广昌路32号</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>0757-22611036</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr"/>
+      <c r="G344" t="inlineStr"/>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>明日之星蒙特梭利实验园(金榜分园)</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Foshan</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>广东省佛山市顺德区大良街道金榜民安路21号</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>0757-22203273</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr"/>
+      <c r="G345" t="inlineStr"/>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>蒙特梭利蒙曦幼儿园(复地新城店)</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Wuxi</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>江苏省无锡市惠山区政和大道99号复地新城37-6号</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>19941586777</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr"/>
+      <c r="G346" t="inlineStr"/>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>宜兴市湖畔乐蒙幼儿园</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Wuxi</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>江苏省无锡市宜兴市洑溪河公园F幢</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>18306152051</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr"/>
+      <c r="G347" t="inlineStr"/>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>无锡市锡山区乐蒙幼儿园</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Wuxi</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>江苏省无锡市锡山区胶阳东路588号</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>4006585597</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr"/>
+      <c r="G348" t="inlineStr"/>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>恒大城琪蒙幼儿园</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Nanchang</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Jiangxi</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>江西省南昌市南昌县恒大城</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>13576011788</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr"/>
+      <c r="G349" t="inlineStr"/>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>国际蒙特梭利亲幼园</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Taiyuan</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Shanxi</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>太原市娄烦镇南大街</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr"/>
+      <c r="G350" t="inlineStr"/>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>金泽蒙特梭利园</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Taiyuan</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Shanxi</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>太原市小店区荣军北街清枫华景</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="inlineStr"/>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>Baidu Maps Tier-2</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I303"/>
@@ -32597,6 +34205,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="12">
       <c r="A3" s="19" t="inlineStr">
         <is>
@@ -32684,6 +34293,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="15" customHeight="1" s="12">
       <c r="A9" s="20" t="inlineStr">
         <is>
@@ -32961,6 +34571,7 @@
         <v>1</v>
       </c>
     </row>
+    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="12">
       <c r="A38" s="20" t="inlineStr">
         <is>

</xml_diff>